<commit_message>
Record the age-band, median, and adjusted smoking results.
These are the figures the resume cites, computed from the same 1,338-policy file.
</commit_message>
<xml_diff>
--- a/output/policies.xlsx
+++ b/output/policies.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="policies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="age bands" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="policies" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -652,6 +653,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Average charges by age band</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>age band</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>smoker</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>policies</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>average charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>18-29</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C4">
+        <f>COUNTIFS(Policies[smoker],"yes",Policies[age],"&gt;=18",Policies[age],"&lt;=29")</f>
+        <v/>
+      </c>
+      <c r="D4" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"yes",Policies[age],"&gt;=18",Policies[age],"&lt;=29")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>18-29</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C5">
+        <f>COUNTIFS(Policies[smoker],"no",Policies[age],"&gt;=18",Policies[age],"&lt;=29")</f>
+        <v/>
+      </c>
+      <c r="D5" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"no",Policies[age],"&gt;=18",Policies[age],"&lt;=29")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30-44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(Policies[smoker],"yes",Policies[age],"&gt;=30",Policies[age],"&lt;=44")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"yes",Policies[age],"&gt;=30",Policies[age],"&lt;=44")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>30-44</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS(Policies[smoker],"no",Policies[age],"&gt;=30",Policies[age],"&lt;=44")</f>
+        <v/>
+      </c>
+      <c r="D7" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"no",Policies[age],"&gt;=30",Policies[age],"&lt;=44")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>45-64</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS(Policies[smoker],"yes",Policies[age],"&gt;=45",Policies[age],"&lt;=64")</f>
+        <v/>
+      </c>
+      <c r="D8" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"yes",Policies[age],"&gt;=45",Policies[age],"&lt;=64")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>45-64</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>COUNTIFS(Policies[smoker],"no",Policies[age],"&gt;=45",Policies[age],"&lt;=64")</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>AVERAGEIFS(Policies[charges],Policies[smoker],"no",Policies[age],"&gt;=45",Policies[age],"&lt;=64")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G1339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>